<commit_message>
feat(brain): complete Phase 1 Brain integration
</commit_message>
<xml_diff>
--- a/ARCHITECTURE_HANDBOOK_v1.0.xlsx
+++ b/ARCHITECTURE_HANDBOOK_v1.0.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6930" tabRatio="939" firstSheet="1" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6930" tabRatio="939" firstSheet="12" activeTab="17"/>
   </bookViews>
   <sheets>
     <sheet name="BOT Architecture" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,8 @@
     <sheet name="13 DEVELOPMENT WORKFLOW" sheetId="14" r:id="rId15"/>
     <sheet name="14" sheetId="15" r:id="rId16"/>
     <sheet name="TRADING_PHILOSOPHY" sheetId="16" r:id="rId17"/>
-    <sheet name="The Sailing Principle" sheetId="17" r:id="rId18"/>
+    <sheet name="Brain constitution" sheetId="29" r:id="rId18"/>
+    <sheet name="The Sailing Principle" sheetId="17" r:id="rId19"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BOT Architecture'!$A$1:$H$1</definedName>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1249" uniqueCount="753">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1493" uniqueCount="942">
   <si>
     <t>Module</t>
   </si>
@@ -2380,6 +2381,657 @@
   </si>
   <si>
     <t>The market decides.</t>
+  </si>
+  <si>
+    <t>---</t>
+  </si>
+  <si>
+    <t># Long-Term Brain Behaviour (Approved)</t>
+  </si>
+  <si>
+    <t>These are approved design principles for future development. They are not immediate implementation tasks.</t>
+  </si>
+  <si>
+    <t>## Position Intelligence</t>
+  </si>
+  <si>
+    <t>The Brain should continue evaluating existing positions after entry, not only before entry.</t>
+  </si>
+  <si>
+    <t>When important new information arrives, it should determine whether it changes the quality of the original trade.</t>
+  </si>
+  <si>
+    <t>Examples include:</t>
+  </si>
+  <si>
+    <t>• Financial results</t>
+  </si>
+  <si>
+    <t>• Major corporate announcements</t>
+  </si>
+  <si>
+    <t>• Government policies</t>
+  </si>
+  <si>
+    <t>• Regulatory actions</t>
+  </si>
+  <si>
+    <t>• Sector-wide developments</t>
+  </si>
+  <si>
+    <t>• Macro events</t>
+  </si>
+  <si>
+    <t>• Global events</t>
+  </si>
+  <si>
+    <t>The Brain should decide whether the new information is:</t>
+  </si>
+  <si>
+    <t>• Strongly Positive</t>
+  </si>
+  <si>
+    <t>• Mildly Positive</t>
+  </si>
+  <si>
+    <t>• Neutral</t>
+  </si>
+  <si>
+    <t>• Mildly Negative</t>
+  </si>
+  <si>
+    <t>• Strongly Negative</t>
+  </si>
+  <si>
+    <t>Desired behaviour:</t>
+  </si>
+  <si>
+    <t>Strongly Positive</t>
+  </si>
+  <si>
+    <t>• Consider increasing conviction.</t>
+  </si>
+  <si>
+    <t>• Allow larger trailing profits.</t>
+  </si>
+  <si>
+    <t>• Extend profit expectations when supported by market behaviour.</t>
+  </si>
+  <si>
+    <t>Mildly Positive</t>
+  </si>
+  <si>
+    <t>• Continue observing.</t>
+  </si>
+  <si>
+    <t>• Avoid immediate position changes.</t>
+  </si>
+  <si>
+    <t>Neutral</t>
+  </si>
+  <si>
+    <t>• No action.</t>
+  </si>
+  <si>
+    <t>Mildly Negative</t>
+  </si>
+  <si>
+    <t>• Tighten risk management.</t>
+  </si>
+  <si>
+    <t>• Increase monitoring.</t>
+  </si>
+  <si>
+    <t>Strongly Negative</t>
+  </si>
+  <si>
+    <t>• Consider reducing exposure or exiting if market behaviour confirms deterioration.</t>
+  </si>
+  <si>
+    <t>The Brain should never react to news alone.</t>
+  </si>
+  <si>
+    <t>It must combine:</t>
+  </si>
+  <si>
+    <t>• Price action</t>
+  </si>
+  <si>
+    <t>• Volume</t>
+  </si>
+  <si>
+    <t>• Market regime</t>
+  </si>
+  <si>
+    <t>• Sector strength</t>
+  </si>
+  <si>
+    <t>• Historical behaviour</t>
+  </si>
+  <si>
+    <t>• Existing evidence</t>
+  </si>
+  <si>
+    <t>• Confidence score</t>
+  </si>
+  <si>
+    <t>before changing any position management decision.</t>
+  </si>
+  <si>
+    <t>## Market Behaviour First</t>
+  </si>
+  <si>
+    <t>Future discussions about sectors, themes, industries and position management should always begin with how markets actually behave.</t>
+  </si>
+  <si>
+    <t>Implementation should follow market understanding—not the other way around.</t>
+  </si>
+  <si>
+    <t>Whenever designing new intelligence, prioritize market structure, institutional behaviour and historical patterns before discussing code.</t>
+  </si>
+  <si>
+    <t>## Portfolio Quality</t>
+  </si>
+  <si>
+    <t>Long-term objective:</t>
+  </si>
+  <si>
+    <t>Reduce avoidable stop-loss exits while allowing high-quality winners to run longer through adaptive intelligence rather than fixed rules.</t>
+  </si>
+  <si>
+    <t>ORB AUTO TRADER CONSTITUTION v1.0</t>
+  </si>
+  <si>
+    <t>Article 1 — Supreme Authority</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The Brain is the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>only</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> component allowed to make trading decisions.</t>
+    </r>
+  </si>
+  <si>
+    <t>No other module may:</t>
+  </si>
+  <si>
+    <t>decide BUY</t>
+  </si>
+  <si>
+    <t>decide SELL</t>
+  </si>
+  <si>
+    <t>decide EXIT</t>
+  </si>
+  <si>
+    <t>decide TARGET</t>
+  </si>
+  <si>
+    <t>decide ADD</t>
+  </si>
+  <si>
+    <t>decide REDUCE</t>
+  </si>
+  <si>
+    <t>decide HOLD</t>
+  </si>
+  <si>
+    <t>Every other component either:</t>
+  </si>
+  <si>
+    <t>observes</t>
+  </si>
+  <si>
+    <t>analyzes</t>
+  </si>
+  <si>
+    <t>validates</t>
+  </si>
+  <si>
+    <t>executes</t>
+  </si>
+  <si>
+    <t>Article 2 — Three Layers</t>
+  </si>
+  <si>
+    <t>Layer 1 — Observation Layer</t>
+  </si>
+  <si>
+    <t>These modules observe markets.</t>
+  </si>
+  <si>
+    <t>Macro Engine</t>
+  </si>
+  <si>
+    <t>Commodity Engine</t>
+  </si>
+  <si>
+    <t>Global Engine</t>
+  </si>
+  <si>
+    <t>Market Story</t>
+  </si>
+  <si>
+    <t>Market Memory</t>
+  </si>
+  <si>
+    <t>Historical Data</t>
+  </si>
+  <si>
+    <t>Output:</t>
+  </si>
+  <si>
+    <t>Observations</t>
+  </si>
+  <si>
+    <t>Nothing else.</t>
+  </si>
+  <si>
+    <t>No decisions.</t>
+  </si>
+  <si>
+    <t>Layer 2 — Intelligence Layer</t>
+  </si>
+  <si>
+    <t>Evidence Builder</t>
+  </si>
+  <si>
+    <t>Evidence Validator</t>
+  </si>
+  <si>
+    <t>Conviction Engine</t>
+  </si>
+  <si>
+    <t>Output</t>
+  </si>
+  <si>
+    <t>Evidence</t>
+  </si>
+  <si>
+    <t>Confidence</t>
+  </si>
+  <si>
+    <t>Conviction</t>
+  </si>
+  <si>
+    <t>Still no decisions.</t>
+  </si>
+  <si>
+    <t>Layer 3 — Decision Layer</t>
+  </si>
+  <si>
+    <t>Only</t>
+  </si>
+  <si>
+    <t>Brain</t>
+  </si>
+  <si>
+    <t>Receives</t>
+  </si>
+  <si>
+    <t>Everything</t>
+  </si>
+  <si>
+    <t>Produces</t>
+  </si>
+  <si>
+    <t>BUY</t>
+  </si>
+  <si>
+    <t>WAIT</t>
+  </si>
+  <si>
+    <t>IGNORE</t>
+  </si>
+  <si>
+    <t>ADD</t>
+  </si>
+  <si>
+    <t>REDUCE</t>
+  </si>
+  <si>
+    <t>EXIT</t>
+  </si>
+  <si>
+    <t>Capital Tier</t>
+  </si>
+  <si>
+    <t>Entry Mode</t>
+  </si>
+  <si>
+    <t>Target Mode</t>
+  </si>
+  <si>
+    <t>Exit Mode</t>
+  </si>
+  <si>
+    <t>Reasons</t>
+  </si>
+  <si>
+    <t>Warnings</t>
+  </si>
+  <si>
+    <t>Article 3 — Execution Layer</t>
+  </si>
+  <si>
+    <t>These modules obey.</t>
+  </si>
+  <si>
+    <t>Trade Selection Engine</t>
+  </si>
+  <si>
+    <t>Portfolio Risk Manager</t>
+  </si>
+  <si>
+    <t>Broker</t>
+  </si>
+  <si>
+    <t>Telegram</t>
+  </si>
+  <si>
+    <t>Trade Logger</t>
+  </si>
+  <si>
+    <t>None of them think.</t>
+  </si>
+  <si>
+    <t>Article 4 — Brain Responsibilities</t>
+  </si>
+  <si>
+    <t>Brain decides</t>
+  </si>
+  <si>
+    <t>Entry</t>
+  </si>
+  <si>
+    <t>Existing Position</t>
+  </si>
+  <si>
+    <t>HOLD</t>
+  </si>
+  <si>
+    <t>Capital</t>
+  </si>
+  <si>
+    <t>NONE</t>
+  </si>
+  <si>
+    <t>LOW</t>
+  </si>
+  <si>
+    <t>MEDIUM</t>
+  </si>
+  <si>
+    <t>HIGH</t>
+  </si>
+  <si>
+    <t>FULL</t>
+  </si>
+  <si>
+    <t>FIXED</t>
+  </si>
+  <si>
+    <t>DYNAMIC</t>
+  </si>
+  <si>
+    <t>TRAIL</t>
+  </si>
+  <si>
+    <t>QUICK EXIT</t>
+  </si>
+  <si>
+    <t>Increase</t>
+  </si>
+  <si>
+    <t>Maintain</t>
+  </si>
+  <si>
+    <t>Reduce</t>
+  </si>
+  <si>
+    <t>Too many IT stocks?</t>
+  </si>
+  <si>
+    <t>Brain decides.</t>
+  </si>
+  <si>
+    <t>Too much PSU exposure?</t>
+  </si>
+  <si>
+    <t>Good results?</t>
+  </si>
+  <si>
+    <t>Bad government policy?</t>
+  </si>
+  <si>
+    <t>Global event?</t>
+  </si>
+  <si>
+    <t>Article 5 — Information Flow</t>
+  </si>
+  <si>
+    <t>This is where the current code needs to evolve.</t>
+  </si>
+  <si>
+    <t>Current</t>
+  </si>
+  <si>
+    <t>Tick</t>
+  </si>
+  <si>
+    <t>Observation Layer</t>
+  </si>
+  <si>
+    <t>Evidence Layer</t>
+  </si>
+  <si>
+    <t>Decision</t>
+  </si>
+  <si>
+    <t>Notice something.</t>
+  </si>
+  <si>
+    <t>Trade Selection disappears as a decision maker.</t>
+  </si>
+  <si>
+    <t>It becomes</t>
+  </si>
+  <si>
+    <t>Decision Router</t>
+  </si>
+  <si>
+    <t>That is a huge simplification.</t>
+  </si>
+  <si>
+    <t>Article 6 — Brain Never Sleeps</t>
+  </si>
+  <si>
+    <t>This is probably the most important rule.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The Brain is </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>not called only at entry</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>It runs continuously.</t>
+  </si>
+  <si>
+    <t>Still evaluating.</t>
+  </si>
+  <si>
+    <t>The Brain never stops thinking.</t>
+  </si>
+  <si>
+    <t>Every new piece of evidence updates its understanding of:</t>
+  </si>
+  <si>
+    <t>Market</t>
+  </si>
+  <si>
+    <t>Positions</t>
+  </si>
+  <si>
+    <t>Opportunities</t>
+  </si>
+  <si>
+    <t>Risk</t>
+  </si>
+  <si>
+    <t>Capital allocation</t>
+  </si>
+  <si>
+    <t>Article 7 — The Brain Has Memory</t>
+  </si>
+  <si>
+    <t>This was always your long-term vision.</t>
+  </si>
+  <si>
+    <t>The Brain remembers.</t>
+  </si>
+  <si>
+    <t>Not just today's news.</t>
+  </si>
+  <si>
+    <t>It remembers:</t>
+  </si>
+  <si>
+    <t>similar RBI cycles</t>
+  </si>
+  <si>
+    <t>similar election periods</t>
+  </si>
+  <si>
+    <t>similar result seasons</t>
+  </si>
+  <si>
+    <t>similar commodity shocks</t>
+  </si>
+  <si>
+    <t>similar tariff announcements</t>
+  </si>
+  <si>
+    <t>similar market rotations</t>
+  </si>
+  <si>
+    <t>Eventually it should say:</t>
+  </si>
+  <si>
+    <t>"This setup has occurred seven times before. The average winner was +8.4%, with IT and Capital Goods leading while FMCG lagged."</t>
+  </si>
+  <si>
+    <t>That is what transforms the system from an ORB bot into an institutional decision platform.</t>
+  </si>
+  <si>
+    <t>What I want to do next</t>
+  </si>
+  <si>
+    <t>Before we write a single line of integration code, I want to produce one final artifact:</t>
+  </si>
+  <si>
+    <t>Brain Decision Flow (v1)</t>
+  </si>
+  <si>
+    <t>It will specify, in exact sequence:</t>
+  </si>
+  <si>
+    <t>1. What happens when a live tick arrives.</t>
+  </si>
+  <si>
+    <t>2. Which module is called next.</t>
+  </si>
+  <si>
+    <t>3. What data each module produces.</t>
+  </si>
+  <si>
+    <t>4. What the Brain consumes.</t>
+  </si>
+  <si>
+    <t>5. What the Brain returns.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">6. How </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>engine.py</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>trade_selection_engine.py</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> change—with the smallest possible modifications.</t>
+    </r>
+  </si>
+  <si>
+    <t>That document will become our implementation guide. Once it's approved, we can integrate the Brain in a controlled, one-file-at-a-time manner without breaking the architecture we've spent months building. I believe that plan is achievable within this session.</t>
   </si>
 </sst>
 </file>
@@ -2468,7 +3120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2504,11 +3156,15 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="6" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="6" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="20" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -4212,11 +4868,11 @@
       </c>
     </row>
     <row r="17" spans="1:3">
-      <c r="A17" s="13" t="s">
+      <c r="A17" s="15" t="s">
         <v>460</v>
       </c>
-      <c r="B17" s="13"/>
-      <c r="C17" s="13"/>
+      <c r="B17" s="15"/>
+      <c r="C17" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -4902,7 +5558,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A287"/>
+  <dimension ref="A1:A369"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="123" bestFit="1" customWidth="1"/>
@@ -5773,6 +6429,276 @@
         <v>633</v>
       </c>
     </row>
+    <row r="289" spans="1:1">
+      <c r="A289" t="s">
+        <v>753</v>
+      </c>
+    </row>
+    <row r="291" spans="1:1">
+      <c r="A291" t="s">
+        <v>754</v>
+      </c>
+    </row>
+    <row r="293" spans="1:1">
+      <c r="A293" t="s">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="295" spans="1:1">
+      <c r="A295" t="s">
+        <v>756</v>
+      </c>
+    </row>
+    <row r="297" spans="1:1">
+      <c r="A297" t="s">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="299" spans="1:1">
+      <c r="A299" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="301" spans="1:1">
+      <c r="A301" t="s">
+        <v>759</v>
+      </c>
+    </row>
+    <row r="303" spans="1:1">
+      <c r="A303" t="s">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="304" spans="1:1">
+      <c r="A304" t="s">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="305" spans="1:1">
+      <c r="A305" t="s">
+        <v>762</v>
+      </c>
+    </row>
+    <row r="306" spans="1:1">
+      <c r="A306" t="s">
+        <v>763</v>
+      </c>
+    </row>
+    <row r="307" spans="1:1">
+      <c r="A307" t="s">
+        <v>764</v>
+      </c>
+    </row>
+    <row r="308" spans="1:1">
+      <c r="A308" t="s">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="309" spans="1:1">
+      <c r="A309" t="s">
+        <v>766</v>
+      </c>
+    </row>
+    <row r="311" spans="1:1">
+      <c r="A311" t="s">
+        <v>767</v>
+      </c>
+    </row>
+    <row r="313" spans="1:1">
+      <c r="A313" t="s">
+        <v>768</v>
+      </c>
+    </row>
+    <row r="314" spans="1:1">
+      <c r="A314" t="s">
+        <v>769</v>
+      </c>
+    </row>
+    <row r="315" spans="1:1">
+      <c r="A315" t="s">
+        <v>770</v>
+      </c>
+    </row>
+    <row r="316" spans="1:1">
+      <c r="A316" t="s">
+        <v>771</v>
+      </c>
+    </row>
+    <row r="317" spans="1:1">
+      <c r="A317" t="s">
+        <v>772</v>
+      </c>
+    </row>
+    <row r="319" spans="1:1">
+      <c r="A319" t="s">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="321" spans="1:1">
+      <c r="A321" t="s">
+        <v>774</v>
+      </c>
+    </row>
+    <row r="322" spans="1:1">
+      <c r="A322" t="s">
+        <v>775</v>
+      </c>
+    </row>
+    <row r="323" spans="1:1">
+      <c r="A323" t="s">
+        <v>776</v>
+      </c>
+    </row>
+    <row r="324" spans="1:1">
+      <c r="A324" t="s">
+        <v>777</v>
+      </c>
+    </row>
+    <row r="326" spans="1:1">
+      <c r="A326" t="s">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="327" spans="1:1">
+      <c r="A327" t="s">
+        <v>779</v>
+      </c>
+    </row>
+    <row r="328" spans="1:1">
+      <c r="A328" t="s">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="330" spans="1:1">
+      <c r="A330" t="s">
+        <v>781</v>
+      </c>
+    </row>
+    <row r="331" spans="1:1">
+      <c r="A331" t="s">
+        <v>782</v>
+      </c>
+    </row>
+    <row r="333" spans="1:1">
+      <c r="A333" t="s">
+        <v>783</v>
+      </c>
+    </row>
+    <row r="334" spans="1:1">
+      <c r="A334" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="335" spans="1:1">
+      <c r="A335" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="337" spans="1:1">
+      <c r="A337" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="338" spans="1:1">
+      <c r="A338" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="340" spans="1:1">
+      <c r="A340" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="341" spans="1:1">
+      <c r="A341" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="343" spans="1:1">
+      <c r="A343" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="344" spans="1:1">
+      <c r="A344" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="345" spans="1:1">
+      <c r="A345" t="s">
+        <v>792</v>
+      </c>
+    </row>
+    <row r="346" spans="1:1">
+      <c r="A346" t="s">
+        <v>793</v>
+      </c>
+    </row>
+    <row r="347" spans="1:1">
+      <c r="A347" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="348" spans="1:1">
+      <c r="A348" t="s">
+        <v>795</v>
+      </c>
+    </row>
+    <row r="349" spans="1:1">
+      <c r="A349" t="s">
+        <v>796</v>
+      </c>
+    </row>
+    <row r="351" spans="1:1">
+      <c r="A351" t="s">
+        <v>797</v>
+      </c>
+    </row>
+    <row r="353" spans="1:1">
+      <c r="A353" t="s">
+        <v>753</v>
+      </c>
+    </row>
+    <row r="355" spans="1:1">
+      <c r="A355" t="s">
+        <v>798</v>
+      </c>
+    </row>
+    <row r="357" spans="1:1">
+      <c r="A357" t="s">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="359" spans="1:1">
+      <c r="A359" t="s">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="361" spans="1:1">
+      <c r="A361" t="s">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="363" spans="1:1">
+      <c r="A363" t="s">
+        <v>753</v>
+      </c>
+    </row>
+    <row r="365" spans="1:1">
+      <c r="A365" t="s">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="367" spans="1:1">
+      <c r="A367" t="s">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="369" spans="1:1">
+      <c r="A369" t="s">
+        <v>804</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
@@ -5780,6 +6706,1272 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A423"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="220.08984375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" ht="31">
+      <c r="A1" s="9" t="s">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" ht="23.5">
+      <c r="A3" s="7" t="s">
+        <v>806</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1">
+      <c r="A5" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1">
+      <c r="A7" t="s">
+        <v>808</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1">
+      <c r="A8" s="11"/>
+    </row>
+    <row r="9" spans="1:1">
+      <c r="A9" s="11" t="s">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1">
+      <c r="A10" s="11"/>
+    </row>
+    <row r="11" spans="1:1">
+      <c r="A11" s="11" t="s">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1">
+      <c r="A12" s="11"/>
+    </row>
+    <row r="13" spans="1:1">
+      <c r="A13" s="11" t="s">
+        <v>811</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1">
+      <c r="A14" s="11"/>
+    </row>
+    <row r="15" spans="1:1">
+      <c r="A15" s="11" t="s">
+        <v>812</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1">
+      <c r="A16" s="11"/>
+    </row>
+    <row r="17" spans="1:1">
+      <c r="A17" s="11" t="s">
+        <v>813</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1">
+      <c r="A18" s="11"/>
+    </row>
+    <row r="19" spans="1:1">
+      <c r="A19" s="11" t="s">
+        <v>814</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1">
+      <c r="A20" s="11"/>
+    </row>
+    <row r="21" spans="1:1">
+      <c r="A21" s="11" t="s">
+        <v>815</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1">
+      <c r="A23" t="s">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1">
+      <c r="A24" s="11"/>
+    </row>
+    <row r="25" spans="1:1">
+      <c r="A25" s="11" t="s">
+        <v>817</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1">
+      <c r="A26" s="11"/>
+    </row>
+    <row r="27" spans="1:1">
+      <c r="A27" s="11" t="s">
+        <v>818</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1">
+      <c r="A28" s="11"/>
+    </row>
+    <row r="29" spans="1:1">
+      <c r="A29" s="11" t="s">
+        <v>819</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1">
+      <c r="A30" s="11"/>
+    </row>
+    <row r="31" spans="1:1">
+      <c r="A31" s="11" t="s">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" ht="31">
+      <c r="A35" s="9" t="s">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" ht="23.5">
+      <c r="A37" s="7" t="s">
+        <v>822</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1">
+      <c r="A39" t="s">
+        <v>823</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1">
+      <c r="A41" s="10" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1">
+      <c r="A42" s="5"/>
+    </row>
+    <row r="43" spans="1:1">
+      <c r="A43" s="10" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1">
+      <c r="A44" s="5"/>
+    </row>
+    <row r="45" spans="1:1">
+      <c r="A45" s="10" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1">
+      <c r="A46" s="5"/>
+    </row>
+    <row r="47" spans="1:1">
+      <c r="A47" s="10" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1">
+      <c r="A48" s="5"/>
+    </row>
+    <row r="49" spans="1:1">
+      <c r="A49" s="10" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1">
+      <c r="A50" s="5"/>
+    </row>
+    <row r="51" spans="1:1">
+      <c r="A51" s="10" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1">
+      <c r="A52" s="5"/>
+    </row>
+    <row r="53" spans="1:1">
+      <c r="A53" s="10" t="s">
+        <v>824</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1">
+      <c r="A54" s="5"/>
+    </row>
+    <row r="55" spans="1:1">
+      <c r="A55" s="10" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1">
+      <c r="A56" s="5"/>
+    </row>
+    <row r="57" spans="1:1">
+      <c r="A57" s="10" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1">
+      <c r="A58" s="5"/>
+    </row>
+    <row r="59" spans="1:1">
+      <c r="A59" s="10" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1">
+      <c r="A60" s="5"/>
+    </row>
+    <row r="61" spans="1:1">
+      <c r="A61" s="10" t="s">
+        <v>828</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1">
+      <c r="A62" s="5"/>
+    </row>
+    <row r="63" spans="1:1">
+      <c r="A63" s="10" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1">
+      <c r="A64" s="5"/>
+    </row>
+    <row r="65" spans="1:1">
+      <c r="A65" s="10" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1">
+      <c r="A66" s="5"/>
+    </row>
+    <row r="67" spans="1:1">
+      <c r="A67" s="10" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1">
+      <c r="A68" s="5"/>
+    </row>
+    <row r="69" spans="1:1">
+      <c r="A69" s="10" t="s">
+        <v>829</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1">
+      <c r="A71" t="s">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1">
+      <c r="A73" s="10" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1">
+      <c r="A75" t="s">
+        <v>832</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1">
+      <c r="A77" t="s">
+        <v>833</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" ht="23.5">
+      <c r="A81" s="7" t="s">
+        <v>834</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1">
+      <c r="A83" s="10" t="s">
+        <v>835</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1">
+      <c r="A84" s="5"/>
+    </row>
+    <row r="85" spans="1:1">
+      <c r="A85" s="10" t="s">
+        <v>836</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1">
+      <c r="A86" s="5"/>
+    </row>
+    <row r="87" spans="1:1">
+      <c r="A87" s="10" t="s">
+        <v>837</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1">
+      <c r="A89" t="s">
+        <v>838</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1">
+      <c r="A91" s="10" t="s">
+        <v>839</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1">
+      <c r="A92" s="5"/>
+    </row>
+    <row r="93" spans="1:1">
+      <c r="A93" s="10" t="s">
+        <v>840</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1">
+      <c r="A94" s="5"/>
+    </row>
+    <row r="95" spans="1:1">
+      <c r="A95" s="10" t="s">
+        <v>841</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1">
+      <c r="A97" t="s">
+        <v>842</v>
+      </c>
+    </row>
+    <row r="101" spans="1:1" ht="23.5">
+      <c r="A101" s="7" t="s">
+        <v>843</v>
+      </c>
+    </row>
+    <row r="103" spans="1:1">
+      <c r="A103" t="s">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="105" spans="1:1">
+      <c r="A105" s="10" t="s">
+        <v>845</v>
+      </c>
+    </row>
+    <row r="107" spans="1:1">
+      <c r="A107" t="s">
+        <v>846</v>
+      </c>
+    </row>
+    <row r="109" spans="1:1">
+      <c r="A109" s="10" t="s">
+        <v>847</v>
+      </c>
+    </row>
+    <row r="111" spans="1:1">
+      <c r="A111" t="s">
+        <v>848</v>
+      </c>
+    </row>
+    <row r="113" spans="1:1">
+      <c r="A113" s="10" t="s">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="114" spans="1:1">
+      <c r="A114" s="5"/>
+    </row>
+    <row r="115" spans="1:1">
+      <c r="A115" s="10" t="s">
+        <v>850</v>
+      </c>
+    </row>
+    <row r="116" spans="1:1">
+      <c r="A116" s="5"/>
+    </row>
+    <row r="117" spans="1:1">
+      <c r="A117" s="10" t="s">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="118" spans="1:1">
+      <c r="A118" s="5"/>
+    </row>
+    <row r="119" spans="1:1">
+      <c r="A119" s="10" t="s">
+        <v>852</v>
+      </c>
+    </row>
+    <row r="120" spans="1:1">
+      <c r="A120" s="5"/>
+    </row>
+    <row r="121" spans="1:1">
+      <c r="A121" s="10" t="s">
+        <v>853</v>
+      </c>
+    </row>
+    <row r="122" spans="1:1">
+      <c r="A122" s="5"/>
+    </row>
+    <row r="123" spans="1:1">
+      <c r="A123" s="10" t="s">
+        <v>854</v>
+      </c>
+    </row>
+    <row r="124" spans="1:1">
+      <c r="A124" s="5"/>
+    </row>
+    <row r="125" spans="1:1">
+      <c r="A125" s="10" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="126" spans="1:1">
+      <c r="A126" s="5"/>
+    </row>
+    <row r="127" spans="1:1">
+      <c r="A127" s="10" t="s">
+        <v>856</v>
+      </c>
+    </row>
+    <row r="128" spans="1:1">
+      <c r="A128" s="5"/>
+    </row>
+    <row r="129" spans="1:1">
+      <c r="A129" s="10" t="s">
+        <v>857</v>
+      </c>
+    </row>
+    <row r="130" spans="1:1">
+      <c r="A130" s="5"/>
+    </row>
+    <row r="131" spans="1:1">
+      <c r="A131" s="10" t="s">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="132" spans="1:1">
+      <c r="A132" s="5"/>
+    </row>
+    <row r="133" spans="1:1">
+      <c r="A133" s="10" t="s">
+        <v>840</v>
+      </c>
+    </row>
+    <row r="134" spans="1:1">
+      <c r="A134" s="5"/>
+    </row>
+    <row r="135" spans="1:1">
+      <c r="A135" s="10" t="s">
+        <v>859</v>
+      </c>
+    </row>
+    <row r="136" spans="1:1">
+      <c r="A136" s="5"/>
+    </row>
+    <row r="137" spans="1:1">
+      <c r="A137" s="10" t="s">
+        <v>860</v>
+      </c>
+    </row>
+    <row r="141" spans="1:1" ht="31">
+      <c r="A141" s="9" t="s">
+        <v>861</v>
+      </c>
+    </row>
+    <row r="143" spans="1:1">
+      <c r="A143" t="s">
+        <v>862</v>
+      </c>
+    </row>
+    <row r="145" spans="1:1">
+      <c r="A145" s="10" t="s">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="146" spans="1:1">
+      <c r="A146" s="5"/>
+    </row>
+    <row r="147" spans="1:1">
+      <c r="A147" s="10" t="s">
+        <v>864</v>
+      </c>
+    </row>
+    <row r="148" spans="1:1">
+      <c r="A148" s="5"/>
+    </row>
+    <row r="149" spans="1:1">
+      <c r="A149" s="10" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="150" spans="1:1">
+      <c r="A150" s="5"/>
+    </row>
+    <row r="151" spans="1:1">
+      <c r="A151" s="10" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="152" spans="1:1">
+      <c r="A152" s="5"/>
+    </row>
+    <row r="153" spans="1:1">
+      <c r="A153" s="10" t="s">
+        <v>865</v>
+      </c>
+    </row>
+    <row r="154" spans="1:1">
+      <c r="A154" s="5"/>
+    </row>
+    <row r="155" spans="1:1">
+      <c r="A155" s="10" t="s">
+        <v>866</v>
+      </c>
+    </row>
+    <row r="156" spans="1:1">
+      <c r="A156" s="5"/>
+    </row>
+    <row r="157" spans="1:1">
+      <c r="A157" s="10" t="s">
+        <v>867</v>
+      </c>
+    </row>
+    <row r="159" spans="1:1">
+      <c r="A159" t="s">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="163" spans="1:1" ht="31">
+      <c r="A163" s="9" t="s">
+        <v>869</v>
+      </c>
+    </row>
+    <row r="165" spans="1:1">
+      <c r="A165" t="s">
+        <v>870</v>
+      </c>
+    </row>
+    <row r="167" spans="1:1" ht="17.5">
+      <c r="A167" s="8" t="s">
+        <v>871</v>
+      </c>
+    </row>
+    <row r="169" spans="1:1">
+      <c r="A169" t="s">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="171" spans="1:1">
+      <c r="A171" t="s">
+        <v>850</v>
+      </c>
+    </row>
+    <row r="173" spans="1:1">
+      <c r="A173" t="s">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="177" spans="1:1" ht="17.5">
+      <c r="A177" s="8" t="s">
+        <v>872</v>
+      </c>
+    </row>
+    <row r="179" spans="1:1">
+      <c r="A179" t="s">
+        <v>873</v>
+      </c>
+    </row>
+    <row r="181" spans="1:1">
+      <c r="A181" t="s">
+        <v>852</v>
+      </c>
+    </row>
+    <row r="183" spans="1:1">
+      <c r="A183" t="s">
+        <v>853</v>
+      </c>
+    </row>
+    <row r="185" spans="1:1">
+      <c r="A185" t="s">
+        <v>854</v>
+      </c>
+    </row>
+    <row r="189" spans="1:1" ht="17.5">
+      <c r="A189" s="8" t="s">
+        <v>874</v>
+      </c>
+    </row>
+    <row r="191" spans="1:1">
+      <c r="A191" t="s">
+        <v>875</v>
+      </c>
+    </row>
+    <row r="193" spans="1:1">
+      <c r="A193" t="s">
+        <v>876</v>
+      </c>
+    </row>
+    <row r="195" spans="1:1">
+      <c r="A195" t="s">
+        <v>877</v>
+      </c>
+    </row>
+    <row r="197" spans="1:1">
+      <c r="A197" t="s">
+        <v>878</v>
+      </c>
+    </row>
+    <row r="199" spans="1:1">
+      <c r="A199" t="s">
+        <v>879</v>
+      </c>
+    </row>
+    <row r="203" spans="1:1" ht="17.5">
+      <c r="A203" s="8" t="s">
+        <v>678</v>
+      </c>
+    </row>
+    <row r="205" spans="1:1">
+      <c r="A205" t="s">
+        <v>880</v>
+      </c>
+    </row>
+    <row r="207" spans="1:1">
+      <c r="A207" t="s">
+        <v>881</v>
+      </c>
+    </row>
+    <row r="209" spans="1:1">
+      <c r="A209" t="s">
+        <v>882</v>
+      </c>
+    </row>
+    <row r="211" spans="1:1">
+      <c r="A211" t="s">
+        <v>883</v>
+      </c>
+    </row>
+    <row r="215" spans="1:1" ht="17.5">
+      <c r="A215" s="8" t="s">
+        <v>840</v>
+      </c>
+    </row>
+    <row r="217" spans="1:1">
+      <c r="A217" t="s">
+        <v>884</v>
+      </c>
+    </row>
+    <row r="219" spans="1:1">
+      <c r="A219" t="s">
+        <v>885</v>
+      </c>
+    </row>
+    <row r="221" spans="1:1">
+      <c r="A221" t="s">
+        <v>886</v>
+      </c>
+    </row>
+    <row r="225" spans="1:1" ht="17.5">
+      <c r="A225" s="8" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="227" spans="1:1">
+      <c r="A227" t="s">
+        <v>887</v>
+      </c>
+    </row>
+    <row r="229" spans="1:1">
+      <c r="A229" t="s">
+        <v>888</v>
+      </c>
+    </row>
+    <row r="231" spans="1:1">
+      <c r="A231" t="s">
+        <v>889</v>
+      </c>
+    </row>
+    <row r="233" spans="1:1">
+      <c r="A233" t="s">
+        <v>888</v>
+      </c>
+    </row>
+    <row r="237" spans="1:1" ht="17.5">
+      <c r="A237" s="8" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="239" spans="1:1">
+      <c r="A239" t="s">
+        <v>890</v>
+      </c>
+    </row>
+    <row r="241" spans="1:1">
+      <c r="A241" t="s">
+        <v>888</v>
+      </c>
+    </row>
+    <row r="243" spans="1:1">
+      <c r="A243" t="s">
+        <v>891</v>
+      </c>
+    </row>
+    <row r="245" spans="1:1">
+      <c r="A245" t="s">
+        <v>888</v>
+      </c>
+    </row>
+    <row r="247" spans="1:1">
+      <c r="A247" t="s">
+        <v>892</v>
+      </c>
+    </row>
+    <row r="249" spans="1:1">
+      <c r="A249" t="s">
+        <v>888</v>
+      </c>
+    </row>
+    <row r="253" spans="1:1" ht="31">
+      <c r="A253" s="9" t="s">
+        <v>893</v>
+      </c>
+    </row>
+    <row r="255" spans="1:1">
+      <c r="A255" t="s">
+        <v>894</v>
+      </c>
+    </row>
+    <row r="257" spans="1:1">
+      <c r="A257" t="s">
+        <v>895</v>
+      </c>
+    </row>
+    <row r="259" spans="1:1">
+      <c r="A259" s="10" t="s">
+        <v>896</v>
+      </c>
+    </row>
+    <row r="260" spans="1:1">
+      <c r="A260" s="5"/>
+    </row>
+    <row r="261" spans="1:1">
+      <c r="A261" s="10" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="262" spans="1:1">
+      <c r="A262" s="5"/>
+    </row>
+    <row r="263" spans="1:1">
+      <c r="A263" s="10" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="264" spans="1:1">
+      <c r="A264" s="5"/>
+    </row>
+    <row r="265" spans="1:1">
+      <c r="A265" s="10" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="266" spans="1:1">
+      <c r="A266" s="5"/>
+    </row>
+    <row r="267" spans="1:1">
+      <c r="A267" s="10" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="268" spans="1:1">
+      <c r="A268" s="5"/>
+    </row>
+    <row r="269" spans="1:1">
+      <c r="A269" s="10" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="270" spans="1:1">
+      <c r="A270" s="5"/>
+    </row>
+    <row r="271" spans="1:1">
+      <c r="A271" s="10" t="s">
+        <v>839</v>
+      </c>
+    </row>
+    <row r="272" spans="1:1">
+      <c r="A272" s="5"/>
+    </row>
+    <row r="273" spans="1:1">
+      <c r="A273" s="10" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="274" spans="1:1">
+      <c r="A274" s="5"/>
+    </row>
+    <row r="275" spans="1:1">
+      <c r="A275" s="10" t="s">
+        <v>841</v>
+      </c>
+    </row>
+    <row r="276" spans="1:1">
+      <c r="A276" s="5"/>
+    </row>
+    <row r="277" spans="1:1">
+      <c r="A277" s="10" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="278" spans="1:1">
+      <c r="A278" s="5"/>
+    </row>
+    <row r="279" spans="1:1">
+      <c r="A279" s="10" t="s">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="281" spans="1:1">
+      <c r="A281" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="283" spans="1:1">
+      <c r="A283" s="10" t="s">
+        <v>896</v>
+      </c>
+    </row>
+    <row r="284" spans="1:1">
+      <c r="A284" s="5"/>
+    </row>
+    <row r="285" spans="1:1">
+      <c r="A285" s="10" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="286" spans="1:1">
+      <c r="A286" s="5"/>
+    </row>
+    <row r="287" spans="1:1">
+      <c r="A287" s="10" t="s">
+        <v>897</v>
+      </c>
+    </row>
+    <row r="288" spans="1:1">
+      <c r="A288" s="5"/>
+    </row>
+    <row r="289" spans="1:1">
+      <c r="A289" s="10" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="290" spans="1:1">
+      <c r="A290" s="5"/>
+    </row>
+    <row r="291" spans="1:1">
+      <c r="A291" s="10" t="s">
+        <v>898</v>
+      </c>
+    </row>
+    <row r="292" spans="1:1">
+      <c r="A292" s="5"/>
+    </row>
+    <row r="293" spans="1:1">
+      <c r="A293" s="10" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="294" spans="1:1">
+      <c r="A294" s="5"/>
+    </row>
+    <row r="295" spans="1:1">
+      <c r="A295" s="10" t="s">
+        <v>845</v>
+      </c>
+    </row>
+    <row r="296" spans="1:1">
+      <c r="A296" s="5"/>
+    </row>
+    <row r="297" spans="1:1">
+      <c r="A297" s="10" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="298" spans="1:1">
+      <c r="A298" s="5"/>
+    </row>
+    <row r="299" spans="1:1">
+      <c r="A299" s="10" t="s">
+        <v>899</v>
+      </c>
+    </row>
+    <row r="300" spans="1:1">
+      <c r="A300" s="5"/>
+    </row>
+    <row r="301" spans="1:1">
+      <c r="A301" s="10" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="302" spans="1:1">
+      <c r="A302" s="5"/>
+    </row>
+    <row r="303" spans="1:1">
+      <c r="A303" s="10" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="304" spans="1:1">
+      <c r="A304" s="5"/>
+    </row>
+    <row r="305" spans="1:1">
+      <c r="A305" s="10" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="306" spans="1:1">
+      <c r="A306" s="5"/>
+    </row>
+    <row r="307" spans="1:1">
+      <c r="A307" s="10" t="s">
+        <v>865</v>
+      </c>
+    </row>
+    <row r="309" spans="1:1">
+      <c r="A309" t="s">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="311" spans="1:1">
+      <c r="A311" t="s">
+        <v>901</v>
+      </c>
+    </row>
+    <row r="313" spans="1:1">
+      <c r="A313" t="s">
+        <v>902</v>
+      </c>
+    </row>
+    <row r="315" spans="1:1">
+      <c r="A315" s="10" t="s">
+        <v>903</v>
+      </c>
+    </row>
+    <row r="317" spans="1:1">
+      <c r="A317" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="321" spans="1:1" ht="31">
+      <c r="A321" s="9" t="s">
+        <v>905</v>
+      </c>
+    </row>
+    <row r="323" spans="1:1">
+      <c r="A323" t="s">
+        <v>906</v>
+      </c>
+    </row>
+    <row r="325" spans="1:1">
+      <c r="A325" t="s">
+        <v>907</v>
+      </c>
+    </row>
+    <row r="327" spans="1:1">
+      <c r="A327" t="s">
+        <v>908</v>
+      </c>
+    </row>
+    <row r="329" spans="1:1">
+      <c r="A329" s="17">
+        <v>0.3888888888888889</v>
+      </c>
+    </row>
+    <row r="330" spans="1:1">
+      <c r="A330" s="5"/>
+    </row>
+    <row r="331" spans="1:1">
+      <c r="A331" s="10" t="s">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="333" spans="1:1">
+      <c r="A333" s="16">
+        <v>0.40625</v>
+      </c>
+    </row>
+    <row r="335" spans="1:1">
+      <c r="A335" t="s">
+        <v>909</v>
+      </c>
+    </row>
+    <row r="337" spans="1:1">
+      <c r="A337" s="16">
+        <v>0.4375</v>
+      </c>
+    </row>
+    <row r="339" spans="1:1">
+      <c r="A339" t="s">
+        <v>909</v>
+      </c>
+    </row>
+    <row r="341" spans="1:1">
+      <c r="A341" s="16">
+        <v>0.46875</v>
+      </c>
+    </row>
+    <row r="343" spans="1:1">
+      <c r="A343" t="s">
+        <v>909</v>
+      </c>
+    </row>
+    <row r="345" spans="1:1">
+      <c r="A345" s="16">
+        <v>0.54513888888888895</v>
+      </c>
+    </row>
+    <row r="347" spans="1:1">
+      <c r="A347" t="s">
+        <v>909</v>
+      </c>
+    </row>
+    <row r="349" spans="1:1">
+      <c r="A349" s="16">
+        <v>0.61111111111111105</v>
+      </c>
+    </row>
+    <row r="351" spans="1:1">
+      <c r="A351" t="s">
+        <v>909</v>
+      </c>
+    </row>
+    <row r="353" spans="1:1">
+      <c r="A353" s="16">
+        <v>0.63194444444444442</v>
+      </c>
+    </row>
+    <row r="355" spans="1:1">
+      <c r="A355" t="s">
+        <v>909</v>
+      </c>
+    </row>
+    <row r="357" spans="1:1">
+      <c r="A357" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="359" spans="1:1">
+      <c r="A359" t="s">
+        <v>911</v>
+      </c>
+    </row>
+    <row r="360" spans="1:1">
+      <c r="A360" s="11"/>
+    </row>
+    <row r="361" spans="1:1">
+      <c r="A361" s="11" t="s">
+        <v>912</v>
+      </c>
+    </row>
+    <row r="362" spans="1:1">
+      <c r="A362" s="11"/>
+    </row>
+    <row r="363" spans="1:1">
+      <c r="A363" s="11" t="s">
+        <v>913</v>
+      </c>
+    </row>
+    <row r="364" spans="1:1">
+      <c r="A364" s="11"/>
+    </row>
+    <row r="365" spans="1:1">
+      <c r="A365" s="11" t="s">
+        <v>914</v>
+      </c>
+    </row>
+    <row r="366" spans="1:1">
+      <c r="A366" s="11"/>
+    </row>
+    <row r="367" spans="1:1">
+      <c r="A367" s="11" t="s">
+        <v>915</v>
+      </c>
+    </row>
+    <row r="368" spans="1:1">
+      <c r="A368" s="11"/>
+    </row>
+    <row r="369" spans="1:1">
+      <c r="A369" s="11" t="s">
+        <v>916</v>
+      </c>
+    </row>
+    <row r="373" spans="1:1" ht="31">
+      <c r="A373" s="9" t="s">
+        <v>917</v>
+      </c>
+    </row>
+    <row r="375" spans="1:1">
+      <c r="A375" t="s">
+        <v>918</v>
+      </c>
+    </row>
+    <row r="377" spans="1:1">
+      <c r="A377" t="s">
+        <v>919</v>
+      </c>
+    </row>
+    <row r="379" spans="1:1">
+      <c r="A379" t="s">
+        <v>920</v>
+      </c>
+    </row>
+    <row r="381" spans="1:1">
+      <c r="A381" t="s">
+        <v>921</v>
+      </c>
+    </row>
+    <row r="382" spans="1:1">
+      <c r="A382" s="11"/>
+    </row>
+    <row r="383" spans="1:1">
+      <c r="A383" s="11" t="s">
+        <v>922</v>
+      </c>
+    </row>
+    <row r="384" spans="1:1">
+      <c r="A384" s="11"/>
+    </row>
+    <row r="385" spans="1:1">
+      <c r="A385" s="11" t="s">
+        <v>923</v>
+      </c>
+    </row>
+    <row r="386" spans="1:1">
+      <c r="A386" s="11"/>
+    </row>
+    <row r="387" spans="1:1">
+      <c r="A387" s="11" t="s">
+        <v>924</v>
+      </c>
+    </row>
+    <row r="388" spans="1:1">
+      <c r="A388" s="11"/>
+    </row>
+    <row r="389" spans="1:1">
+      <c r="A389" s="11" t="s">
+        <v>925</v>
+      </c>
+    </row>
+    <row r="390" spans="1:1">
+      <c r="A390" s="11"/>
+    </row>
+    <row r="391" spans="1:1">
+      <c r="A391" s="11" t="s">
+        <v>926</v>
+      </c>
+    </row>
+    <row r="392" spans="1:1">
+      <c r="A392" s="11"/>
+    </row>
+    <row r="393" spans="1:1">
+      <c r="A393" s="11" t="s">
+        <v>927</v>
+      </c>
+    </row>
+    <row r="395" spans="1:1">
+      <c r="A395" t="s">
+        <v>928</v>
+      </c>
+    </row>
+    <row r="396" spans="1:1">
+      <c r="A396" s="11"/>
+    </row>
+    <row r="397" spans="1:1">
+      <c r="A397" s="11" t="s">
+        <v>929</v>
+      </c>
+    </row>
+    <row r="399" spans="1:1">
+      <c r="A399" t="s">
+        <v>930</v>
+      </c>
+    </row>
+    <row r="403" spans="1:1" ht="31">
+      <c r="A403" s="9" t="s">
+        <v>931</v>
+      </c>
+    </row>
+    <row r="405" spans="1:1">
+      <c r="A405" t="s">
+        <v>932</v>
+      </c>
+    </row>
+    <row r="406" spans="1:1">
+      <c r="A406" s="11"/>
+    </row>
+    <row r="407" spans="1:1">
+      <c r="A407" s="12" t="s">
+        <v>933</v>
+      </c>
+    </row>
+    <row r="409" spans="1:1">
+      <c r="A409" t="s">
+        <v>934</v>
+      </c>
+    </row>
+    <row r="410" spans="1:1">
+      <c r="A410" s="11"/>
+    </row>
+    <row r="411" spans="1:1">
+      <c r="A411" s="11" t="s">
+        <v>935</v>
+      </c>
+    </row>
+    <row r="412" spans="1:1">
+      <c r="A412" s="11"/>
+    </row>
+    <row r="413" spans="1:1">
+      <c r="A413" s="11" t="s">
+        <v>936</v>
+      </c>
+    </row>
+    <row r="414" spans="1:1">
+      <c r="A414" s="11"/>
+    </row>
+    <row r="415" spans="1:1">
+      <c r="A415" s="11" t="s">
+        <v>937</v>
+      </c>
+    </row>
+    <row r="416" spans="1:1">
+      <c r="A416" s="11"/>
+    </row>
+    <row r="417" spans="1:1">
+      <c r="A417" s="11" t="s">
+        <v>938</v>
+      </c>
+    </row>
+    <row r="418" spans="1:1">
+      <c r="A418" s="11"/>
+    </row>
+    <row r="419" spans="1:1">
+      <c r="A419" s="11" t="s">
+        <v>939</v>
+      </c>
+    </row>
+    <row r="420" spans="1:1">
+      <c r="A420" s="11"/>
+    </row>
+    <row r="421" spans="1:1">
+      <c r="A421" s="11" t="s">
+        <v>940</v>
+      </c>
+    </row>
+    <row r="423" spans="1:1">
+      <c r="A423" t="s">
+        <v>941</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:A19"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
@@ -6037,7 +8229,7 @@
       </c>
     </row>
     <row r="3" spans="1:1">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="13" t="s">
         <v>644</v>
       </c>
     </row>
@@ -6067,7 +8259,7 @@
       </c>
     </row>
     <row r="17" spans="1:1">
-      <c r="A17" s="14" t="s">
+      <c r="A17" s="13" t="s">
         <v>649</v>
       </c>
     </row>
@@ -6110,7 +8302,7 @@
       </c>
     </row>
     <row r="32" spans="1:1">
-      <c r="A32" s="14" t="s">
+      <c r="A32" s="13" t="s">
         <v>656</v>
       </c>
     </row>
@@ -6168,7 +8360,7 @@
       </c>
     </row>
     <row r="51" spans="1:1">
-      <c r="A51" s="14" t="s">
+      <c r="A51" s="13" t="s">
         <v>666</v>
       </c>
     </row>
@@ -6219,7 +8411,7 @@
       </c>
     </row>
     <row r="71" spans="1:1">
-      <c r="A71" s="14" t="s">
+      <c r="A71" s="13" t="s">
         <v>675</v>
       </c>
     </row>
@@ -6380,7 +8572,7 @@
       </c>
     </row>
     <row r="117" spans="1:1">
-      <c r="A117" s="14" t="s">
+      <c r="A117" s="13" t="s">
         <v>690</v>
       </c>
     </row>
@@ -6406,7 +8598,7 @@
       <c r="A124" s="5"/>
     </row>
     <row r="125" spans="1:1">
-      <c r="A125" s="15">
+      <c r="A125" s="14">
         <v>30000</v>
       </c>
     </row>
@@ -6468,7 +8660,7 @@
       </c>
     </row>
     <row r="147" spans="1:1">
-      <c r="A147" s="14" t="s">
+      <c r="A147" s="13" t="s">
         <v>703</v>
       </c>
     </row>
@@ -6618,7 +8810,7 @@
       <c r="A204" s="5"/>
     </row>
     <row r="205" spans="1:1">
-      <c r="A205" s="15">
+      <c r="A205" s="14">
         <v>42000</v>
       </c>
     </row>

</xml_diff>